<commit_message>
Updated ESP model - 2025-09-22 22:49
</commit_message>
<xml_diff>
--- a/VerveStacks_ESP/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ESP/ReportDefs_vervestacks.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\VerveStacks\assumptions\VerveStacks_ISO_template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FBFA3B6F-77C9-4026-A7F7-2B3175ECC1C9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EB1C8A7-4808-4116-B649-64C70DAF59A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ScenMap_OLD" sheetId="70" r:id="rId1"/>
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="845" uniqueCount="418">
   <si>
     <t>Unit</t>
   </si>
@@ -867,9 +867,6 @@
     <t>ar6_r10</t>
   </si>
   <si>
-    <t>ELC,ELC_???-???*,e[_]*</t>
-  </si>
-  <si>
     <t>*ccs</t>
   </si>
   <si>
@@ -1239,13 +1236,106 @@
     <t>g64</t>
   </si>
   <si>
-    <t>f97p50</t>
-  </si>
-  <si>
     <t>f96p10</t>
   </si>
   <si>
     <t>f96p90</t>
+  </si>
+  <si>
+    <t>f96p50</t>
+  </si>
+  <si>
+    <t>ELC,ELC_???[_]???*,e[_]*</t>
+  </si>
+  <si>
+    <t>IRE</t>
+  </si>
+  <si>
+    <t>g[_]*</t>
+  </si>
+  <si>
+    <t>Grid Capacity</t>
+  </si>
+  <si>
+    <t>Grid New Capacity</t>
+  </si>
+  <si>
+    <t>Sector</t>
+  </si>
+  <si>
+    <t>e_dem*</t>
+  </si>
+  <si>
+    <t>Industry and Buildings</t>
+  </si>
+  <si>
+    <t>ev_bat*</t>
+  </si>
+  <si>
+    <t>H2Prd*</t>
+  </si>
+  <si>
+    <t>e_dem*,ev_bat*,H2Prd*</t>
+  </si>
+  <si>
+    <t>e*</t>
+  </si>
+  <si>
+    <t>~tradeflow_exp</t>
+  </si>
+  <si>
+    <t>Internal variable to create Grid-level trade flows</t>
+  </si>
+  <si>
+    <t>p,c</t>
+  </si>
+  <si>
+    <t>~tradeflow_imp</t>
+  </si>
+  <si>
+    <t>ELC_???[_]???*,e[_]*</t>
+  </si>
+  <si>
+    <t>VerveStacks</t>
+  </si>
+  <si>
+    <t>Tech_origin</t>
+  </si>
+  <si>
+    <t>ep_*</t>
+  </si>
+  <si>
+    <t>GEM_operating</t>
+  </si>
+  <si>
+    <t>en_pc_*</t>
+  </si>
+  <si>
+    <t>GEM_pre-constr</t>
+  </si>
+  <si>
+    <t>ep_m_*</t>
+  </si>
+  <si>
+    <t>GEM_mothballed</t>
+  </si>
+  <si>
+    <t>en_a_*</t>
+  </si>
+  <si>
+    <t>GEM_announced</t>
+  </si>
+  <si>
+    <t>en_can_*</t>
+  </si>
+  <si>
+    <t>GEM_cancelled</t>
+  </si>
+  <si>
+    <t>en_she_*</t>
+  </si>
+  <si>
+    <t>GEM_shelved</t>
   </si>
 </sst>
 </file>
@@ -2311,10 +2401,10 @@
         <v>11</v>
       </c>
       <c r="T16" t="s">
+        <v>262</v>
+      </c>
+      <c r="U16" t="s">
         <v>263</v>
-      </c>
-      <c r="U16" t="s">
-        <v>264</v>
       </c>
     </row>
     <row r="17" spans="1:17">
@@ -3821,7 +3911,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{10ADB714-E6AA-4E3E-B77B-62B65BA0E218}">
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="14.86328125" bestFit="1" customWidth="1"/>
@@ -4427,7 +4517,7 @@
         <v>69</v>
       </c>
       <c r="B50" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C50" t="s">
         <v>132</v>
@@ -4441,7 +4531,7 @@
         <v>69</v>
       </c>
       <c r="B51" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C51" t="s">
         <v>133</v>
@@ -4509,6 +4599,116 @@
       </c>
       <c r="C56" t="s">
         <v>114</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5">
+      <c r="A57" t="s">
+        <v>392</v>
+      </c>
+      <c r="B57" t="s">
+        <v>393</v>
+      </c>
+      <c r="C57" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5">
+      <c r="A58" t="s">
+        <v>392</v>
+      </c>
+      <c r="B58" t="s">
+        <v>395</v>
+      </c>
+      <c r="C58" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5">
+      <c r="A59" t="s">
+        <v>392</v>
+      </c>
+      <c r="B59" t="s">
+        <v>396</v>
+      </c>
+      <c r="C59" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5">
+      <c r="A60" t="s">
+        <v>405</v>
+      </c>
+      <c r="B60" t="s">
+        <v>120</v>
+      </c>
+      <c r="C60" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5">
+      <c r="A61" t="s">
+        <v>405</v>
+      </c>
+      <c r="B61" t="s">
+        <v>406</v>
+      </c>
+      <c r="C61" t="s">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5">
+      <c r="A62" t="s">
+        <v>405</v>
+      </c>
+      <c r="B62" t="s">
+        <v>408</v>
+      </c>
+      <c r="C62" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5">
+      <c r="A63" t="s">
+        <v>405</v>
+      </c>
+      <c r="B63" t="s">
+        <v>410</v>
+      </c>
+      <c r="C63" t="s">
+        <v>411</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5">
+      <c r="A64" t="s">
+        <v>405</v>
+      </c>
+      <c r="B64" t="s">
+        <v>412</v>
+      </c>
+      <c r="C64" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3">
+      <c r="A65" t="s">
+        <v>405</v>
+      </c>
+      <c r="B65" t="s">
+        <v>414</v>
+      </c>
+      <c r="C65" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3">
+      <c r="A66" t="s">
+        <v>405</v>
+      </c>
+      <c r="B66" t="s">
+        <v>416</v>
+      </c>
+      <c r="C66" t="s">
+        <v>417</v>
       </c>
     </row>
   </sheetData>
@@ -4773,7 +4973,7 @@
         <v>63</v>
       </c>
       <c r="O4" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
     </row>
     <row r="5" spans="2:24">
@@ -4801,19 +5001,19 @@
         <v>sg_timeslice</v>
       </c>
       <c r="N5" t="s">
+        <v>296</v>
+      </c>
+      <c r="O5" t="s">
         <v>297</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>298</v>
-      </c>
-      <c r="P5" t="s">
-        <v>299</v>
       </c>
       <c r="Q5" t="s">
         <v>124</v>
       </c>
       <c r="R5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
     </row>
     <row r="6" spans="2:24">
@@ -4844,7 +5044,7 @@
         <v>5</v>
       </c>
       <c r="O6" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="P6">
         <v>1</v>
@@ -4853,16 +5053,16 @@
         <v>238</v>
       </c>
       <c r="R6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="T6" t="s">
         <v>238</v>
       </c>
       <c r="U6" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="W6" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="X6" t="s">
         <v>258</v>
@@ -4896,7 +5096,7 @@
         <v>5</v>
       </c>
       <c r="O7" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="P7">
         <v>2</v>
@@ -4905,16 +5105,16 @@
         <v>238</v>
       </c>
       <c r="R7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="T7" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="U7" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="W7" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="X7" t="s">
         <v>257</v>
@@ -4948,7 +5148,7 @@
         <v>5</v>
       </c>
       <c r="O8" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="P8">
         <v>3</v>
@@ -4957,16 +5157,16 @@
         <v>238</v>
       </c>
       <c r="R8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="T8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="U8" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="W8" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="X8" t="s">
         <v>256</v>
@@ -5000,7 +5200,7 @@
         <v>5</v>
       </c>
       <c r="O9" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="P9">
         <v>4</v>
@@ -5009,16 +5209,16 @@
         <v>238</v>
       </c>
       <c r="R9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="T9" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="U9" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="W9" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="X9" t="s">
         <v>255</v>
@@ -5052,7 +5252,7 @@
         <v>5</v>
       </c>
       <c r="O10" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="P10">
         <v>5</v>
@@ -5061,16 +5261,16 @@
         <v>238</v>
       </c>
       <c r="R10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="T10" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="U10" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
       <c r="W10" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="X10" t="s">
         <v>259</v>
@@ -5101,22 +5301,22 @@
         <v>5</v>
       </c>
       <c r="O11" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="P11">
         <v>6</v>
       </c>
       <c r="Q11" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R11" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="T11" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="U11" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="12" spans="2:24">
@@ -5144,22 +5344,22 @@
         <v>5</v>
       </c>
       <c r="O12" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="P12">
         <v>7</v>
       </c>
       <c r="Q12" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="T12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="U12" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
     </row>
     <row r="13" spans="2:24">
@@ -5187,22 +5387,22 @@
         <v>5</v>
       </c>
       <c r="O13" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="P13">
         <v>8</v>
       </c>
       <c r="Q13" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R13" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="T13" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="U13" t="s">
-        <v>386</v>
+        <v>384</v>
       </c>
     </row>
     <row r="14" spans="2:24">
@@ -5230,22 +5430,22 @@
         <v>5</v>
       </c>
       <c r="O14" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="P14">
         <v>9</v>
       </c>
       <c r="Q14" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R14" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="T14" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="U14" t="s">
-        <v>387</v>
+        <v>385</v>
       </c>
     </row>
     <row r="15" spans="2:24">
@@ -5273,16 +5473,16 @@
         <v>5</v>
       </c>
       <c r="O15" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="P15">
         <v>10</v>
       </c>
       <c r="Q15" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="R15" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="T15" t="s">
         <v>230</v>
@@ -5316,16 +5516,16 @@
         <v>5</v>
       </c>
       <c r="O16" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="P16">
         <v>11</v>
       </c>
       <c r="Q16" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R16" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="T16" t="s">
         <v>231</v>
@@ -5359,16 +5559,16 @@
         <v>5</v>
       </c>
       <c r="O17" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="P17">
         <v>12</v>
       </c>
       <c r="Q17" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R17" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="T17" t="s">
         <v>237</v>
@@ -5402,16 +5602,16 @@
         <v>5</v>
       </c>
       <c r="O18" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="P18">
         <v>13</v>
       </c>
       <c r="Q18" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R18" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="T18" t="s">
         <v>232</v>
@@ -5445,16 +5645,16 @@
         <v>5</v>
       </c>
       <c r="O19" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="P19">
         <v>14</v>
       </c>
       <c r="Q19" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R19" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="T19" t="s">
         <v>233</v>
@@ -5488,16 +5688,16 @@
         <v>5</v>
       </c>
       <c r="O20" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="P20">
         <v>15</v>
       </c>
       <c r="Q20" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="R20" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="21" spans="2:21">
@@ -5525,16 +5725,16 @@
         <v>5</v>
       </c>
       <c r="O21" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="P21">
         <v>16</v>
       </c>
       <c r="Q21" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R21" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="22" spans="2:21">
@@ -5562,16 +5762,16 @@
         <v>5</v>
       </c>
       <c r="O22" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="P22">
         <v>17</v>
       </c>
       <c r="Q22" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R22" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="23" spans="2:21">
@@ -5599,16 +5799,16 @@
         <v>5</v>
       </c>
       <c r="O23" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="P23">
         <v>18</v>
       </c>
       <c r="Q23" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R23" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="2:21">
@@ -5636,16 +5836,16 @@
         <v>5</v>
       </c>
       <c r="O24" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="P24">
         <v>19</v>
       </c>
       <c r="Q24" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R24" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="25" spans="2:21">
@@ -5673,16 +5873,16 @@
         <v>5</v>
       </c>
       <c r="O25" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="P25">
         <v>20</v>
       </c>
       <c r="Q25" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="R25" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="26" spans="2:21">
@@ -5710,16 +5910,16 @@
         <v>5</v>
       </c>
       <c r="O26" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="P26">
         <v>21</v>
       </c>
       <c r="Q26" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R26" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="27" spans="2:21">
@@ -5747,16 +5947,16 @@
         <v>5</v>
       </c>
       <c r="O27" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="P27">
         <v>22</v>
       </c>
       <c r="Q27" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R27" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="28" spans="2:21">
@@ -5784,16 +5984,16 @@
         <v>5</v>
       </c>
       <c r="O28" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="P28">
         <v>23</v>
       </c>
       <c r="Q28" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R28" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" spans="2:21">
@@ -5821,16 +6021,16 @@
         <v>5</v>
       </c>
       <c r="O29" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="P29">
         <v>24</v>
       </c>
       <c r="Q29" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R29" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="30" spans="2:21">
@@ -5858,16 +6058,16 @@
         <v>5</v>
       </c>
       <c r="O30" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="P30">
         <v>25</v>
       </c>
       <c r="Q30" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="R30" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" spans="2:21">
@@ -5895,16 +6095,16 @@
         <v>5</v>
       </c>
       <c r="O31" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="P31">
         <v>26</v>
       </c>
       <c r="Q31" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R31" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="32" spans="2:21">
@@ -5932,16 +6132,16 @@
         <v>5</v>
       </c>
       <c r="O32" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="P32">
         <v>27</v>
       </c>
       <c r="Q32" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R32" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="33" spans="2:18">
@@ -5969,16 +6169,16 @@
         <v>5</v>
       </c>
       <c r="O33" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="P33">
         <v>28</v>
       </c>
       <c r="Q33" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R33" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="34" spans="2:18">
@@ -6006,16 +6206,16 @@
         <v>5</v>
       </c>
       <c r="O34" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="P34">
         <v>29</v>
       </c>
       <c r="Q34" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R34" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="35" spans="2:18">
@@ -6043,16 +6243,16 @@
         <v>5</v>
       </c>
       <c r="O35" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="P35">
         <v>30</v>
       </c>
       <c r="Q35" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="R35" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="36" spans="2:18">
@@ -6062,11 +6262,11 @@
       </c>
       <c r="C36" t="str">
         <f t="shared" si="5"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="H36" t="str">
         <f t="shared" si="2"/>
-        <v>e 1.5 deg no OS.f97p50</v>
+        <v>e 1.5 deg no OS.f96p50</v>
       </c>
       <c r="I36" t="str">
         <f t="shared" si="3"/>
@@ -6074,22 +6274,22 @@
       </c>
       <c r="J36" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N36">
         <v>5</v>
       </c>
       <c r="O36" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="P36">
         <v>31</v>
       </c>
       <c r="Q36" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R36" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="37" spans="2:18">
@@ -6099,11 +6299,11 @@
       </c>
       <c r="C37" t="str">
         <f t="shared" si="5"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="H37" t="str">
         <f t="shared" si="2"/>
-        <v>d 1.5 deg OS.f97p50</v>
+        <v>d 1.5 deg OS.f96p50</v>
       </c>
       <c r="I37" t="str">
         <f t="shared" si="3"/>
@@ -6111,22 +6311,22 @@
       </c>
       <c r="J37" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N37">
         <v>5</v>
       </c>
       <c r="O37" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="P37">
         <v>32</v>
       </c>
       <c r="Q37" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R37" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="2:18">
@@ -6136,11 +6336,11 @@
       </c>
       <c r="C38" t="str">
         <f t="shared" si="5"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="H38" t="str">
         <f t="shared" si="2"/>
-        <v>c 2 deg (67%).f97p50</v>
+        <v>c 2 deg (67%).f96p50</v>
       </c>
       <c r="I38" t="str">
         <f t="shared" si="3"/>
@@ -6148,22 +6348,22 @@
       </c>
       <c r="J38" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N38">
         <v>5</v>
       </c>
       <c r="O38" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="P38">
         <v>33</v>
       </c>
       <c r="Q38" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R38" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="39" spans="2:18">
@@ -6173,11 +6373,11 @@
       </c>
       <c r="C39" t="str">
         <f t="shared" si="5"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="H39" t="str">
         <f t="shared" si="2"/>
-        <v>b 2 deg (50%).f97p50</v>
+        <v>b 2 deg (50%).f96p50</v>
       </c>
       <c r="I39" t="str">
         <f t="shared" si="3"/>
@@ -6185,22 +6385,22 @@
       </c>
       <c r="J39" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N39">
         <v>5</v>
       </c>
       <c r="O39" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="P39">
         <v>34</v>
       </c>
       <c r="Q39" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R39" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="40" spans="2:18">
@@ -6210,11 +6410,11 @@
       </c>
       <c r="C40" t="str">
         <f t="shared" si="5"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="H40" t="str">
         <f t="shared" si="2"/>
-        <v>a 3 deg.f97p50</v>
+        <v>a 3 deg.f96p50</v>
       </c>
       <c r="I40" t="str">
         <f t="shared" si="3"/>
@@ -6222,22 +6422,22 @@
       </c>
       <c r="J40" t="str">
         <f t="shared" si="4"/>
-        <v>f97p50</v>
+        <v>f96p50</v>
       </c>
       <c r="N40">
         <v>5</v>
       </c>
       <c r="O40" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="P40">
         <v>35</v>
       </c>
       <c r="Q40" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="R40" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="41" spans="2:18">
@@ -6265,16 +6465,16 @@
         <v>5</v>
       </c>
       <c r="O41" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="P41">
         <v>36</v>
       </c>
       <c r="Q41" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R41" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="42" spans="2:18">
@@ -6302,16 +6502,16 @@
         <v>5</v>
       </c>
       <c r="O42" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="P42">
         <v>37</v>
       </c>
       <c r="Q42" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R42" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="43" spans="2:18">
@@ -6339,16 +6539,16 @@
         <v>5</v>
       </c>
       <c r="O43" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="P43">
         <v>38</v>
       </c>
       <c r="Q43" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R43" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="44" spans="2:18">
@@ -6376,16 +6576,16 @@
         <v>5</v>
       </c>
       <c r="O44" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="P44">
         <v>39</v>
       </c>
       <c r="Q44" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R44" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="45" spans="2:18">
@@ -6413,16 +6613,16 @@
         <v>5</v>
       </c>
       <c r="O45" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="P45">
         <v>40</v>
       </c>
       <c r="Q45" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="R45" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="46" spans="2:18">
@@ -6450,16 +6650,16 @@
         <v>5</v>
       </c>
       <c r="O46" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="P46">
         <v>41</v>
       </c>
       <c r="Q46" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R46" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="47" spans="2:18">
@@ -6487,16 +6687,16 @@
         <v>5</v>
       </c>
       <c r="O47" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="P47">
         <v>42</v>
       </c>
       <c r="Q47" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R47" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="48" spans="2:18">
@@ -6524,16 +6724,16 @@
         <v>5</v>
       </c>
       <c r="O48" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="P48">
         <v>43</v>
       </c>
       <c r="Q48" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R48" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49" spans="2:18">
@@ -6561,16 +6761,16 @@
         <v>5</v>
       </c>
       <c r="O49" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="P49">
         <v>44</v>
       </c>
       <c r="Q49" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R49" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="50" spans="2:18">
@@ -6598,16 +6798,16 @@
         <v>5</v>
       </c>
       <c r="O50" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="P50">
         <v>45</v>
       </c>
       <c r="Q50" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="R50" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="51" spans="2:18">
@@ -6635,7 +6835,7 @@
         <v>5</v>
       </c>
       <c r="O51" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="P51">
         <v>46</v>
@@ -6644,7 +6844,7 @@
         <v>230</v>
       </c>
       <c r="R51" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="52" spans="2:18">
@@ -6672,7 +6872,7 @@
         <v>5</v>
       </c>
       <c r="O52" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="P52">
         <v>47</v>
@@ -6681,7 +6881,7 @@
         <v>230</v>
       </c>
       <c r="R52" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="53" spans="2:18">
@@ -6709,7 +6909,7 @@
         <v>5</v>
       </c>
       <c r="O53" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="P53">
         <v>48</v>
@@ -6718,7 +6918,7 @@
         <v>230</v>
       </c>
       <c r="R53" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="54" spans="2:18">
@@ -6746,7 +6946,7 @@
         <v>5</v>
       </c>
       <c r="O54" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="P54">
         <v>49</v>
@@ -6755,7 +6955,7 @@
         <v>230</v>
       </c>
       <c r="R54" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="55" spans="2:18">
@@ -6783,7 +6983,7 @@
         <v>5</v>
       </c>
       <c r="O55" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="P55">
         <v>50</v>
@@ -6792,7 +6992,7 @@
         <v>230</v>
       </c>
       <c r="R55" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="56" spans="2:18">
@@ -6820,7 +7020,7 @@
         <v>5</v>
       </c>
       <c r="O56" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="P56">
         <v>51</v>
@@ -6829,7 +7029,7 @@
         <v>231</v>
       </c>
       <c r="R56" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="57" spans="2:18">
@@ -6857,7 +7057,7 @@
         <v>5</v>
       </c>
       <c r="O57" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="P57">
         <v>52</v>
@@ -6866,7 +7066,7 @@
         <v>231</v>
       </c>
       <c r="R57" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="58" spans="2:18">
@@ -6894,7 +7094,7 @@
         <v>5</v>
       </c>
       <c r="O58" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="P58">
         <v>53</v>
@@ -6903,7 +7103,7 @@
         <v>231</v>
       </c>
       <c r="R58" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="59" spans="2:18">
@@ -6931,7 +7131,7 @@
         <v>5</v>
       </c>
       <c r="O59" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="P59">
         <v>54</v>
@@ -6940,7 +7140,7 @@
         <v>231</v>
       </c>
       <c r="R59" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="60" spans="2:18">
@@ -6968,7 +7168,7 @@
         <v>5</v>
       </c>
       <c r="O60" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="P60">
         <v>55</v>
@@ -6977,7 +7177,7 @@
         <v>231</v>
       </c>
       <c r="R60" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="61" spans="2:18">
@@ -7005,7 +7205,7 @@
         <v>5</v>
       </c>
       <c r="O61" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="P61">
         <v>56</v>
@@ -7014,7 +7214,7 @@
         <v>237</v>
       </c>
       <c r="R61" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="62" spans="2:18">
@@ -7042,7 +7242,7 @@
         <v>5</v>
       </c>
       <c r="O62" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="P62">
         <v>57</v>
@@ -7051,7 +7251,7 @@
         <v>237</v>
       </c>
       <c r="R62" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="63" spans="2:18">
@@ -7079,7 +7279,7 @@
         <v>5</v>
       </c>
       <c r="O63" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="P63">
         <v>58</v>
@@ -7088,7 +7288,7 @@
         <v>237</v>
       </c>
       <c r="R63" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="64" spans="2:18">
@@ -7116,7 +7316,7 @@
         <v>5</v>
       </c>
       <c r="O64" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="P64">
         <v>59</v>
@@ -7125,7 +7325,7 @@
         <v>237</v>
       </c>
       <c r="R64" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="65" spans="2:18">
@@ -7153,7 +7353,7 @@
         <v>5</v>
       </c>
       <c r="O65" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="P65">
         <v>60</v>
@@ -7162,7 +7362,7 @@
         <v>237</v>
       </c>
       <c r="R65" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="66" spans="2:18">
@@ -7190,7 +7390,7 @@
         <v>5</v>
       </c>
       <c r="O66" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
       <c r="P66">
         <v>61</v>
@@ -7199,7 +7399,7 @@
         <v>232</v>
       </c>
       <c r="R66" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="67" spans="2:18">
@@ -7227,7 +7427,7 @@
         <v>5</v>
       </c>
       <c r="O67" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="P67">
         <v>62</v>
@@ -7236,7 +7436,7 @@
         <v>232</v>
       </c>
       <c r="R67" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="68" spans="2:18">
@@ -7264,7 +7464,7 @@
         <v>5</v>
       </c>
       <c r="O68" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
       <c r="P68">
         <v>63</v>
@@ -7273,7 +7473,7 @@
         <v>232</v>
       </c>
       <c r="R68" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="69" spans="2:18">
@@ -7301,7 +7501,7 @@
         <v>5</v>
       </c>
       <c r="O69" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="P69">
         <v>64</v>
@@ -7310,7 +7510,7 @@
         <v>232</v>
       </c>
       <c r="R69" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="70" spans="2:18">
@@ -7338,7 +7538,7 @@
         <v>5</v>
       </c>
       <c r="O70" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="P70">
         <v>65</v>
@@ -7347,7 +7547,7 @@
         <v>232</v>
       </c>
       <c r="R70" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
     <row r="71" spans="2:18">
@@ -7375,7 +7575,7 @@
         <v>5</v>
       </c>
       <c r="O71" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
       <c r="P71">
         <v>66</v>
@@ -7384,7 +7584,7 @@
         <v>233</v>
       </c>
       <c r="R71" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="72" spans="2:18">
@@ -7412,7 +7612,7 @@
         <v>5</v>
       </c>
       <c r="O72" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="P72">
         <v>67</v>
@@ -7421,7 +7621,7 @@
         <v>233</v>
       </c>
       <c r="R72" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="73" spans="2:18">
@@ -7449,7 +7649,7 @@
         <v>5</v>
       </c>
       <c r="O73" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="P73">
         <v>68</v>
@@ -7458,7 +7658,7 @@
         <v>233</v>
       </c>
       <c r="R73" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="74" spans="2:18">
@@ -7486,7 +7686,7 @@
         <v>5</v>
       </c>
       <c r="O74" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="P74">
         <v>69</v>
@@ -7495,7 +7695,7 @@
         <v>233</v>
       </c>
       <c r="R74" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="75" spans="2:18">
@@ -7523,7 +7723,7 @@
         <v>5</v>
       </c>
       <c r="O75" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="P75">
         <v>70</v>
@@ -7532,7 +7732,7 @@
         <v>233</v>
       </c>
       <c r="R75" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
     </row>
   </sheetData>
@@ -7548,7 +7748,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet19"/>
-  <dimension ref="A1:U15"/>
+  <dimension ref="A1:U20"/>
   <sheetFormatPr defaultColWidth="9.1328125" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="13.86328125" bestFit="1" customWidth="1"/>
@@ -7685,7 +7885,7 @@
         <v>157</v>
       </c>
       <c r="I5" t="s">
-        <v>261</v>
+        <v>387</v>
       </c>
       <c r="K5" t="s">
         <v>80</v>
@@ -7769,7 +7969,7 @@
         <v>117</v>
       </c>
       <c r="K9" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="N9" t="s">
         <v>82</v>
@@ -7851,13 +8051,13 @@
     </row>
     <row r="14" spans="1:21">
       <c r="A14" s="4" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="K14" t="s">
+        <v>291</v>
+      </c>
+      <c r="N14" t="s">
         <v>292</v>
-      </c>
-      <c r="N14" t="s">
-        <v>293</v>
       </c>
       <c r="Q14" t="s">
         <v>50</v>
@@ -7865,16 +8065,107 @@
     </row>
     <row r="15" spans="1:21">
       <c r="A15" s="4" t="s">
+        <v>290</v>
+      </c>
+      <c r="K15" t="s">
         <v>291</v>
       </c>
-      <c r="K15" t="s">
-        <v>292</v>
-      </c>
       <c r="N15" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="Q15" t="s">
         <v>50</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21">
+      <c r="A16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C16" t="s">
+        <v>388</v>
+      </c>
+      <c r="D16" t="s">
+        <v>389</v>
+      </c>
+      <c r="K16" t="s">
+        <v>8</v>
+      </c>
+      <c r="N16" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17">
+      <c r="A17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" t="s">
+        <v>388</v>
+      </c>
+      <c r="D17" t="s">
+        <v>389</v>
+      </c>
+      <c r="K17" t="s">
+        <v>8</v>
+      </c>
+      <c r="N17" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17">
+      <c r="A18" s="4" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" t="s">
+        <v>397</v>
+      </c>
+      <c r="I18" t="s">
+        <v>398</v>
+      </c>
+      <c r="K18" t="s">
+        <v>80</v>
+      </c>
+      <c r="N18" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17">
+      <c r="A19" t="s">
+        <v>161</v>
+      </c>
+      <c r="I19" t="s">
+        <v>403</v>
+      </c>
+      <c r="K19" t="s">
+        <v>80</v>
+      </c>
+      <c r="N19" t="s">
+        <v>399</v>
+      </c>
+      <c r="P19" t="s">
+        <v>400</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17">
+      <c r="A20" t="s">
+        <v>5</v>
+      </c>
+      <c r="I20" t="s">
+        <v>403</v>
+      </c>
+      <c r="K20" t="s">
+        <v>80</v>
+      </c>
+      <c r="N20" t="s">
+        <v>402</v>
+      </c>
+      <c r="P20" t="s">
+        <v>400</v>
+      </c>
+      <c r="Q20" t="s">
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -7976,7 +8267,7 @@
   <sheetData>
     <row r="3" spans="1:19" ht="17.25" thickBot="1">
       <c r="A3" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
     </row>
     <row r="4" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -8084,7 +8375,7 @@
     </row>
     <row r="10" spans="1:19" ht="17.25" thickBot="1">
       <c r="A10" s="5" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
     </row>
     <row r="11" spans="1:19" ht="15" thickTop="1" thickBot="1">
@@ -8151,7 +8442,7 @@
         <v>120</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:19">
@@ -8170,7 +8461,7 @@
         <v>160</v>
       </c>
       <c r="M13" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="S13">
         <v>-1</v>
@@ -8192,7 +8483,7 @@
         <v>160</v>
       </c>
       <c r="M14" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="S14">
         <v>-1</v>
@@ -8203,7 +8494,7 @@
         <v>120</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="16" spans="1:19">
@@ -8222,7 +8513,7 @@
         <v>160</v>
       </c>
       <c r="M16" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="S16">
         <v>-1</v>
@@ -8244,7 +8535,7 @@
         <v>160</v>
       </c>
       <c r="M17" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="S17">
         <v>-1</v>
@@ -8255,7 +8546,7 @@
         <v>120</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" spans="1:19">
@@ -8273,7 +8564,7 @@
         <v>160</v>
       </c>
       <c r="M19" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="S19">
         <v>-1</v>
@@ -8294,7 +8585,7 @@
         <v>160</v>
       </c>
       <c r="M20" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="S20">
         <v>-1</v>
@@ -8314,7 +8605,7 @@
         <v>160</v>
       </c>
       <c r="M23" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="S23">
         <v>-1</v>
@@ -8438,7 +8729,7 @@
         <v>94</v>
       </c>
       <c r="B12" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="13" spans="1:3">
@@ -8446,7 +8737,7 @@
         <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="14" spans="1:3">
@@ -8979,7 +9270,7 @@
         <v>202</v>
       </c>
       <c r="B24" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="25" spans="1:2">
@@ -8987,7 +9278,7 @@
         <v>203</v>
       </c>
       <c r="B25" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="26" spans="1:2">
@@ -9004,7 +9295,7 @@
         <v>187</v>
       </c>
       <c r="B27" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="28" spans="1:2">
@@ -9141,7 +9432,7 @@
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -9150,7 +9441,7 @@
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
@@ -9177,7 +9468,7 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -9186,7 +9477,7 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -9195,18 +9486,18 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="B12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="B13" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
   </sheetData>

</xml_diff>